<commit_message>
chore: Update 2025 pipeline outputs and add manual verification files
- Updated Buckman well production input data (BDW_CHECK)
- Updated Table 1 (ingested data), Table 3 (Rio Pojoaque/Tesuque), Table 4 (Rio Grande/Otowi)
- Added Table 4 and Table 5 manual verification xlsx files for QC review

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/buckman/input/csv/2025/Buckman_Well_Prod_2025_BDW_CHECK.xlsx
+++ b/buckman/input/csv/2025/Buckman_Well_Prod_2025_BDW_CHECK.xlsx
@@ -5,17 +5,30 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\bradwolaver\projects\rg\santafe\buckman\input\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\bradwolaver\projects\rg\santafe\buckman\input\csv\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{48D6027C-E58C-4213-8F74-D9C1CC6FE7EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAE64C4-764B-4431-8A43-6B180BFBA4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{BBA94C1A-76BE-4703-ABCB-2017D30A4558}"/>
+    <workbookView xWindow="28680" yWindow="690" windowWidth="29040" windowHeight="15720" xr2:uid="{BBA94C1A-76BE-4703-ABCB-2017D30A4558}"/>
   </bookViews>
   <sheets>
     <sheet name="Buckman_Well_Prod_2025_BDW_CHEC" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -100,7 +113,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -583,14 +596,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="33" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="16" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -12472,7 +12485,7 @@
       <c r="F245">
         <v>0</v>
       </c>
-      <c r="G245" s="7">
+      <c r="G245" s="12">
         <v>1.698</v>
       </c>
       <c r="H245">
@@ -12519,7 +12532,7 @@
       <c r="F246">
         <v>0</v>
       </c>
-      <c r="G246" s="7">
+      <c r="G246" s="12">
         <v>1.6930000000000001</v>
       </c>
       <c r="H246">
@@ -12566,7 +12579,7 @@
       <c r="F247">
         <v>0</v>
       </c>
-      <c r="G247" s="7">
+      <c r="G247" s="12">
         <v>1.6950000000000001</v>
       </c>
       <c r="H247">
@@ -12613,7 +12626,7 @@
       <c r="F248">
         <v>0</v>
       </c>
-      <c r="G248" s="7">
+      <c r="G248" s="12">
         <v>1.7050000000000001</v>
       </c>
       <c r="H248">
@@ -12660,7 +12673,7 @@
       <c r="F249">
         <v>0</v>
       </c>
-      <c r="G249" s="7">
+      <c r="G249" s="12">
         <v>1.71</v>
       </c>
       <c r="H249">
@@ -12707,7 +12720,7 @@
       <c r="F250">
         <v>0</v>
       </c>
-      <c r="G250" s="7">
+      <c r="G250" s="12">
         <v>1.714</v>
       </c>
       <c r="H250">
@@ -12754,7 +12767,7 @@
       <c r="F251">
         <v>0</v>
       </c>
-      <c r="G251" s="7">
+      <c r="G251" s="12">
         <v>0.48699999999999999</v>
       </c>
       <c r="H251">
@@ -12801,7 +12814,7 @@
       <c r="F252">
         <v>0</v>
       </c>
-      <c r="G252" s="7">
+      <c r="G252" s="12">
         <v>0</v>
       </c>
       <c r="H252">
@@ -12848,7 +12861,7 @@
       <c r="F253">
         <v>0</v>
       </c>
-      <c r="G253" s="7">
+      <c r="G253" s="12">
         <v>0</v>
       </c>
       <c r="H253">
@@ -12895,7 +12908,7 @@
       <c r="F254">
         <v>0</v>
       </c>
-      <c r="G254" s="7">
+      <c r="G254" s="12">
         <v>0</v>
       </c>
       <c r="H254">
@@ -12942,7 +12955,7 @@
       <c r="F255">
         <v>0</v>
       </c>
-      <c r="G255" s="7">
+      <c r="G255" s="12">
         <v>0</v>
       </c>
       <c r="H255">
@@ -12989,7 +13002,7 @@
       <c r="F256">
         <v>0</v>
       </c>
-      <c r="G256" s="7">
+      <c r="G256" s="12">
         <v>0</v>
       </c>
       <c r="H256">
@@ -13036,7 +13049,7 @@
       <c r="F257">
         <v>0</v>
       </c>
-      <c r="G257" s="7">
+      <c r="G257" s="12">
         <v>0</v>
       </c>
       <c r="H257">
@@ -13083,7 +13096,7 @@
       <c r="F258">
         <v>0</v>
       </c>
-      <c r="G258" s="7">
+      <c r="G258" s="12">
         <v>0.436</v>
       </c>
       <c r="H258">
@@ -13130,7 +13143,7 @@
       <c r="F259">
         <v>0</v>
       </c>
-      <c r="G259" s="7">
+      <c r="G259" s="12">
         <v>1.849</v>
       </c>
       <c r="H259">
@@ -13177,7 +13190,7 @@
       <c r="F260">
         <v>0</v>
       </c>
-      <c r="G260" s="7">
+      <c r="G260" s="12">
         <v>0.25700000000000001</v>
       </c>
       <c r="H260">
@@ -13224,7 +13237,7 @@
       <c r="F261">
         <v>0</v>
       </c>
-      <c r="G261" s="7">
+      <c r="G261" s="12">
         <v>1.2E-2</v>
       </c>
       <c r="H261">
@@ -13271,7 +13284,7 @@
       <c r="F262">
         <v>0</v>
       </c>
-      <c r="G262" s="7">
+      <c r="G262" s="12">
         <v>0.30299999999999999</v>
       </c>
       <c r="H262">
@@ -13318,7 +13331,7 @@
       <c r="F263">
         <v>0</v>
       </c>
-      <c r="G263" s="7">
+      <c r="G263" s="12">
         <v>0</v>
       </c>
       <c r="H263">
@@ -13365,7 +13378,7 @@
       <c r="F264">
         <v>0</v>
       </c>
-      <c r="G264" s="7">
+      <c r="G264" s="12">
         <v>0</v>
       </c>
       <c r="H264">
@@ -13412,7 +13425,7 @@
       <c r="F265">
         <v>0</v>
       </c>
-      <c r="G265" s="7">
+      <c r="G265" s="12">
         <v>0</v>
       </c>
       <c r="H265">
@@ -13459,7 +13472,7 @@
       <c r="F266">
         <v>0</v>
       </c>
-      <c r="G266" s="7">
+      <c r="G266" s="12">
         <v>0</v>
       </c>
       <c r="H266">
@@ -13506,7 +13519,7 @@
       <c r="F267">
         <v>0</v>
       </c>
-      <c r="G267" s="7">
+      <c r="G267" s="12">
         <v>0</v>
       </c>
       <c r="H267">
@@ -13553,7 +13566,7 @@
       <c r="F268">
         <v>0</v>
       </c>
-      <c r="G268" s="7">
+      <c r="G268" s="12">
         <v>0</v>
       </c>
       <c r="H268">
@@ -13600,7 +13613,7 @@
       <c r="F269">
         <v>0</v>
       </c>
-      <c r="G269" s="7">
+      <c r="G269" s="12">
         <v>0</v>
       </c>
       <c r="H269">
@@ -13647,7 +13660,7 @@
       <c r="F270">
         <v>0</v>
       </c>
-      <c r="G270" s="7">
+      <c r="G270" s="12">
         <v>3.7999999999999999E-2</v>
       </c>
       <c r="H270">
@@ -13694,7 +13707,7 @@
       <c r="F271">
         <v>0</v>
       </c>
-      <c r="G271" s="7">
+      <c r="G271" s="12">
         <v>0</v>
       </c>
       <c r="H271">
@@ -13741,7 +13754,7 @@
       <c r="F272">
         <v>0</v>
       </c>
-      <c r="G272" s="7">
+      <c r="G272" s="12">
         <v>0</v>
       </c>
       <c r="H272">
@@ -13788,7 +13801,7 @@
       <c r="F273">
         <v>0</v>
       </c>
-      <c r="G273" s="7">
+      <c r="G273" s="12">
         <v>0</v>
       </c>
       <c r="H273">
@@ -13835,7 +13848,7 @@
       <c r="F274">
         <v>0</v>
       </c>
-      <c r="G274" s="7">
+      <c r="G274" s="12">
         <v>0</v>
       </c>
       <c r="H274">
@@ -18427,59 +18440,59 @@
         <v>19</v>
       </c>
       <c r="B372" s="9">
-        <f>SUM(B2:B366)</f>
+        <f t="shared" ref="B372:O372" si="0">SUM(B2:B366)</f>
         <v>162.5019999999999</v>
       </c>
       <c r="C372" s="4">
-        <f>SUM(C2:C366)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D372" s="4">
-        <f>SUM(D2:D366)</f>
+        <f t="shared" si="0"/>
         <v>10.163000000000002</v>
       </c>
       <c r="E372" s="4">
-        <f>SUM(E2:E366)</f>
+        <f t="shared" si="0"/>
         <v>34.02800000000002</v>
       </c>
       <c r="F372" s="4">
-        <f>SUM(F2:F366)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G372" s="9">
-        <f>SUM(G2:G366)</f>
+        <f t="shared" si="0"/>
         <v>71.375999999999976</v>
       </c>
       <c r="H372" s="4">
-        <f>SUM(H2:H366)</f>
+        <f t="shared" si="0"/>
         <v>0.41899999999999998</v>
       </c>
       <c r="I372" s="4">
-        <f>SUM(I2:I366)</f>
+        <f t="shared" si="0"/>
         <v>41.04999999999999</v>
       </c>
       <c r="J372" s="4">
-        <f>SUM(J2:J366)</f>
+        <f t="shared" si="0"/>
         <v>7.6359999999999983</v>
       </c>
       <c r="K372" s="4">
-        <f>SUM(K2:K366)</f>
+        <f t="shared" si="0"/>
         <v>47.307000000000009</v>
       </c>
       <c r="L372" s="4">
-        <f>SUM(L2:L366)</f>
+        <f t="shared" si="0"/>
         <v>26.252000000000006</v>
       </c>
       <c r="M372" s="4">
-        <f>SUM(M2:M366)</f>
+        <f t="shared" si="0"/>
         <v>20.827999999999996</v>
       </c>
       <c r="N372" s="4">
-        <f>SUM(N2:N366)</f>
+        <f t="shared" si="0"/>
         <v>18.964000000000002</v>
       </c>
       <c r="O372" s="4">
-        <f>SUM(O2:O366)</f>
+        <f t="shared" si="0"/>
         <v>440.50849999999997</v>
       </c>
     </row>
@@ -18492,55 +18505,55 @@
         <v>162501999.99999991</v>
       </c>
       <c r="C373" s="5">
-        <f t="shared" ref="C373:O373" si="0">C372*1000000</f>
+        <f t="shared" ref="C373:O373" si="1">C372*1000000</f>
         <v>0</v>
       </c>
       <c r="D373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10163000.000000002</v>
       </c>
       <c r="E373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>34028000.000000022</v>
       </c>
       <c r="F373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G373" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>71375999.99999997</v>
       </c>
       <c r="H373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>419000</v>
       </c>
       <c r="I373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>41049999.999999993</v>
       </c>
       <c r="J373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7635999.9999999981</v>
       </c>
       <c r="K373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>47307000.000000007</v>
       </c>
       <c r="L373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26252000.000000007</v>
       </c>
       <c r="M373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20827999.999999996</v>
       </c>
       <c r="N373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18964000.000000004</v>
       </c>
       <c r="O373" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>440508499.99999994</v>
       </c>
     </row>
@@ -18553,55 +18566,55 @@
         <v>498.70032622272117</v>
       </c>
       <c r="C374" s="6">
-        <f t="shared" ref="C374:O374" si="1">C373/325851</f>
+        <f t="shared" ref="C374:O374" si="2">C373/325851</f>
         <v>0</v>
       </c>
       <c r="D374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>31.189101767372211</v>
       </c>
       <c r="E374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>104.4280975046878</v>
       </c>
       <c r="F374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G374" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>219.04490089028411</v>
       </c>
       <c r="H374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.2858637843677019</v>
       </c>
       <c r="I374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>125.97782422027244</v>
       </c>
       <c r="J374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>23.43402352609014</v>
       </c>
       <c r="K374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>145.17985214100926</v>
       </c>
       <c r="L374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>80.564429754703866</v>
       </c>
       <c r="M374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>63.918784966134815</v>
       </c>
       <c r="N374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>58.198379013721009</v>
       </c>
       <c r="O374" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1351.8709471506913</v>
       </c>
     </row>

</xml_diff>